<commit_message>
Final changes for paper
</commit_message>
<xml_diff>
--- a/Files/Alignment/metadata_fig_4.xlsx
+++ b/Files/Alignment/metadata_fig_4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eugenianikonorova/Desktop/Work/Cornus_sericea_transcriptome_SDH/Files/Alignment/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F4CADF6-0F4E-584A-B804-DF9DD7F65016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F30904A-7793-094D-937E-347EEC207369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="15120" windowHeight="17800" xr2:uid="{103FD404-2B10-9747-BB60-C61F81904F5B}"/>
   </bookViews>
@@ -837,7 +837,7 @@
         <v>0</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>